<commit_message>
workspace and task controller
</commit_message>
<xml_diff>
--- a/Book2.xlsx
+++ b/Book2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ajain\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\saas\saas-backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D5FC1EBB-D107-4B87-9105-3A6E1CB1F715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A62C1424-959B-4D1A-9562-38740055727E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="10300" xr2:uid="{7E5DDFC2-DD2A-4A16-A81F-5518DB3802A1}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="19416" windowHeight="10296" xr2:uid="{7E5DDFC2-DD2A-4A16-A81F-5518DB3802A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,23 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="76">
   <si>
     <t>API Name</t>
   </si>
@@ -74,9 +63,6 @@
     <t>Create Task</t>
   </si>
   <si>
-    <t>POST /workspaces/:workspaceId/tasks</t>
-  </si>
-  <si>
     <t>Create a new task inside workspace</t>
   </si>
   <si>
@@ -104,22 +90,13 @@
     <t>GET /workspaces/:workspaceId/tasks</t>
   </si>
   <si>
-    <t>Get all tasks of workspace</t>
-  </si>
-  <si>
     <t>- workspaceId valid; - workspace exists; - user is member</t>
   </si>
   <si>
-    <t>1. Extract userId; 2. Validate workspaceId; 3. Check membership; 4. Convert 'me'; 5. Apply filters; 6. Fetch tasks; 7. Return response</t>
-  </si>
-  <si>
     <t>401 AuthenticationError; 403 ForbiddenError; 404 NotFoundError; 400 ValidationError; 500 ServerError</t>
   </si>
   <si>
     <t>200 OK</t>
-  </si>
-  <si>
-    <t>workspaceId; - workspace exists; - user is member; - title required; - assignedTo valid member</t>
   </si>
   <si>
     <t>Update Task</t>
@@ -186,16 +163,10 @@
     <t>Authenticated user</t>
   </si>
   <si>
-    <t>Name,</t>
-  </si>
-  <si>
     <t xml:space="preserve">userID must be valid </t>
   </si>
   <si>
     <t>Create a new workspace and assign creator as admin</t>
-  </si>
-  <si>
-    <t>1.set user as admin  3.the workspace with same name must not exist 4. create the worspace</t>
   </si>
   <si>
     <t>Add user to worksapce</t>
@@ -271,13 +242,37 @@
   </si>
   <si>
     <t>Admin/owner</t>
+  </si>
+  <si>
+    <t>workspace ; - user is member; - title required; - assignedTo valid member</t>
+  </si>
+  <si>
+    <t>POST /workspaces/:workspaceId/tasks</t>
+  </si>
+  <si>
+    <t>Get task of workspace based on the filters</t>
+  </si>
+  <si>
+    <t>1. Extract userId; 2. Validate workspaceId; 3. Check membership; ; 5. Apply filters; 6. Fetch tasks; 7. Return response</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> workspaceId valid;taskid is valid I6 - user is member</t>
+  </si>
+  <si>
+    <t>Name,members</t>
+  </si>
+  <si>
+    <t xml:space="preserve">name should be unquie and required ,members must have only valid user </t>
+  </si>
+  <si>
+    <t>1.perform validation, 2set user as owner  3.remove duplicate user entries  4. create the worspace</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -680,20 +675,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3EB739F-88F2-4D69-816F-880D07E0482A}">
   <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="22.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="44.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="48.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.54296875" customWidth="1"/>
+    <col min="1" max="1" width="22.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.09765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.5" customWidth="1"/>
     <col min="5" max="5" width="41" customWidth="1"/>
-    <col min="7" max="7" width="29.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="76.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="107.90625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="105.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.69921875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="76.796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="107.8984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="105.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -728,322 +723,322 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11">
       <c r="A2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" t="s">
-        <v>15</v>
-      </c>
       <c r="F2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H2" t="s">
+        <v>68</v>
+      </c>
+      <c r="I2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>17</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>18</v>
       </c>
-      <c r="K2" t="s">
-        <v>19</v>
-      </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11">
       <c r="A3" s="3"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11">
       <c r="A4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
         <v>20</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" t="s">
         <v>21</v>
       </c>
-      <c r="C4" t="s">
+      <c r="I4" t="s">
+        <v>71</v>
+      </c>
+      <c r="J4" t="s">
         <v>22</v>
       </c>
-      <c r="D4" t="s">
+      <c r="K4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="96.6">
+      <c r="A5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" t="s">
+        <v>72</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="69">
+      <c r="A6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" t="s">
+        <v>73</v>
+      </c>
+      <c r="H7" t="s">
+        <v>74</v>
+      </c>
+      <c r="I7" t="s">
+        <v>75</v>
+      </c>
+      <c r="J7" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" t="s">
         <v>14</v>
       </c>
-      <c r="E4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="F8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" t="s">
         <v>42</v>
       </c>
-      <c r="G4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="I8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J8" t="s">
+        <v>22</v>
+      </c>
+      <c r="K8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I9" t="s">
+        <v>54</v>
+      </c>
+      <c r="J9" t="s">
+        <v>22</v>
+      </c>
+      <c r="K9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s">
+        <v>57</v>
+      </c>
+      <c r="I10" t="s">
+        <v>58</v>
+      </c>
+      <c r="J10" t="s">
+        <v>22</v>
+      </c>
+      <c r="K10" t="s">
         <v>23</v>
       </c>
-      <c r="I4" t="s">
-        <v>24</v>
-      </c>
-      <c r="J4" t="s">
-        <v>25</v>
-      </c>
-      <c r="K4" t="s">
-        <v>26</v>
-      </c>
     </row>
-    <row r="5" spans="1:11" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" t="s">
-        <v>31</v>
-      </c>
-      <c r="H5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="J5" t="s">
-        <v>25</v>
-      </c>
-      <c r="K5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" t="s">
+    <row r="11" spans="1:11" ht="55.2">
+      <c r="A11" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" t="s">
+        <v>61</v>
+      </c>
+      <c r="D11" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" t="s">
+        <v>62</v>
+      </c>
+      <c r="F11" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="I11" t="s">
+        <v>63</v>
+      </c>
+      <c r="J11" t="s">
+        <v>22</v>
+      </c>
+      <c r="K11" t="s">
         <v>39</v>
-      </c>
-      <c r="D6" t="s">
-        <v>37</v>
-      </c>
-      <c r="E6" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" t="s">
-        <v>16</v>
-      </c>
-      <c r="H6" t="s">
-        <v>38</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J6" t="s">
-        <v>25</v>
-      </c>
-      <c r="K6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B7" t="s">
-        <v>53</v>
-      </c>
-      <c r="C7" t="s">
-        <v>48</v>
-      </c>
-      <c r="D7" t="s">
-        <v>45</v>
-      </c>
-      <c r="E7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H7" t="s">
-        <v>47</v>
-      </c>
-      <c r="I7" t="s">
-        <v>49</v>
-      </c>
-      <c r="J7" t="s">
-        <v>25</v>
-      </c>
-      <c r="K7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C8" t="s">
-        <v>51</v>
-      </c>
-      <c r="D8" t="s">
-        <v>73</v>
-      </c>
-      <c r="E8" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" t="s">
-        <v>16</v>
-      </c>
-      <c r="G8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I8" t="s">
-        <v>55</v>
-      </c>
-      <c r="J8" t="s">
-        <v>25</v>
-      </c>
-      <c r="K8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B9" t="s">
-        <v>57</v>
-      </c>
-      <c r="C9" t="s">
-        <v>58</v>
-      </c>
-      <c r="D9" t="s">
-        <v>72</v>
-      </c>
-      <c r="E9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" t="s">
-        <v>16</v>
-      </c>
-      <c r="H9" t="s">
-        <v>59</v>
-      </c>
-      <c r="I9" t="s">
-        <v>60</v>
-      </c>
-      <c r="J9" t="s">
-        <v>25</v>
-      </c>
-      <c r="K9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B10" t="s">
-        <v>62</v>
-      </c>
-      <c r="C10" t="s">
-        <v>65</v>
-      </c>
-      <c r="D10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F10" t="s">
-        <v>16</v>
-      </c>
-      <c r="G10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H10" t="s">
-        <v>63</v>
-      </c>
-      <c r="I10" t="s">
-        <v>64</v>
-      </c>
-      <c r="J10" t="s">
-        <v>25</v>
-      </c>
-      <c r="K10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B11" t="s">
-        <v>70</v>
-      </c>
-      <c r="C11" t="s">
-        <v>67</v>
-      </c>
-      <c r="D11" t="s">
-        <v>73</v>
-      </c>
-      <c r="E11" t="s">
-        <v>68</v>
-      </c>
-      <c r="F11" t="s">
-        <v>16</v>
-      </c>
-      <c r="G11" t="s">
-        <v>16</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="I11" t="s">
-        <v>69</v>
-      </c>
-      <c r="J11" t="s">
-        <v>25</v>
-      </c>
-      <c r="K11" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>